<commit_message>
daily auto push: 2026-09-29 15:42 UTC
</commit_message>
<xml_diff>
--- a/excel/apple3.xlsx
+++ b/excel/apple3.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D4821"/>
+  <dimension ref="A1:D4822"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -86457,7 +86457,7 @@
     <row r="4780">
       <c r="A4780" t="inlineStr">
         <is>
-          <t>2026/12/29</t>
+          <t>2026/09/29</t>
         </is>
       </c>
       <c r="B4780" t="inlineStr">
@@ -86466,10 +86466,10 @@
         </is>
       </c>
       <c r="C4780" t="n">
-        <v>13</v>
+        <v>23</v>
       </c>
       <c r="D4780" t="n">
-        <v>3</v>
+        <v>11</v>
       </c>
     </row>
     <row r="4781">
@@ -86484,7 +86484,7 @@
         </is>
       </c>
       <c r="C4781" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D4781" t="n">
         <v>3</v>
@@ -86502,7 +86502,7 @@
         </is>
       </c>
       <c r="C4782" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D4782" t="n">
         <v>3</v>
@@ -86520,7 +86520,7 @@
         </is>
       </c>
       <c r="C4783" t="n">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="D4783" t="n">
         <v>3</v>
@@ -86529,16 +86529,16 @@
     <row r="4784">
       <c r="A4784" t="inlineStr">
         <is>
-          <t>2026/12/30</t>
+          <t>2026/12/29</t>
         </is>
       </c>
       <c r="B4784" t="inlineStr">
         <is>
-          <t>水</t>
+          <t>火</t>
         </is>
       </c>
       <c r="C4784" t="n">
-        <v>2</v>
+        <v>23</v>
       </c>
       <c r="D4784" t="n">
         <v>3</v>
@@ -86556,7 +86556,7 @@
         </is>
       </c>
       <c r="C4785" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D4785" t="n">
         <v>3</v>
@@ -86574,7 +86574,7 @@
         </is>
       </c>
       <c r="C4786" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="D4786" t="n">
         <v>3</v>
@@ -86592,7 +86592,7 @@
         </is>
       </c>
       <c r="C4787" t="n">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="D4787" t="n">
         <v>3</v>
@@ -86610,7 +86610,7 @@
         </is>
       </c>
       <c r="C4788" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D4788" t="n">
         <v>3</v>
@@ -86628,7 +86628,7 @@
         </is>
       </c>
       <c r="C4789" t="n">
-        <v>22</v>
+        <v>16</v>
       </c>
       <c r="D4789" t="n">
         <v>3</v>
@@ -86637,16 +86637,16 @@
     <row r="4790">
       <c r="A4790" t="inlineStr">
         <is>
-          <t>2026/12/31</t>
+          <t>2026/12/30</t>
         </is>
       </c>
       <c r="B4790" t="inlineStr">
         <is>
-          <t>木</t>
+          <t>水</t>
         </is>
       </c>
       <c r="C4790" t="n">
-        <v>2</v>
+        <v>22</v>
       </c>
       <c r="D4790" t="n">
         <v>3</v>
@@ -86664,7 +86664,7 @@
         </is>
       </c>
       <c r="C4791" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="D4791" t="n">
         <v>3</v>
@@ -86682,7 +86682,7 @@
         </is>
       </c>
       <c r="C4792" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="D4792" t="n">
         <v>3</v>
@@ -86700,7 +86700,7 @@
         </is>
       </c>
       <c r="C4793" t="n">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="D4793" t="n">
         <v>3</v>
@@ -86718,7 +86718,7 @@
         </is>
       </c>
       <c r="C4794" t="n">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="D4794" t="n">
         <v>3</v>
@@ -86736,7 +86736,7 @@
         </is>
       </c>
       <c r="C4795" t="n">
-        <v>22</v>
+        <v>14</v>
       </c>
       <c r="D4795" t="n">
         <v>3</v>
@@ -86745,16 +86745,16 @@
     <row r="4796">
       <c r="A4796" t="inlineStr">
         <is>
-          <t>2027/01/01</t>
+          <t>2026/12/31</t>
         </is>
       </c>
       <c r="B4796" t="inlineStr">
         <is>
-          <t>金</t>
+          <t>木</t>
         </is>
       </c>
       <c r="C4796" t="n">
-        <v>2</v>
+        <v>22</v>
       </c>
       <c r="D4796" t="n">
         <v>3</v>
@@ -86772,7 +86772,7 @@
         </is>
       </c>
       <c r="C4797" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D4797" t="n">
         <v>3</v>
@@ -86790,7 +86790,7 @@
         </is>
       </c>
       <c r="C4798" t="n">
-        <v>13</v>
+        <v>5</v>
       </c>
       <c r="D4798" t="n">
         <v>3</v>
@@ -86808,7 +86808,7 @@
         </is>
       </c>
       <c r="C4799" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D4799" t="n">
         <v>3</v>
@@ -86826,7 +86826,7 @@
         </is>
       </c>
       <c r="C4800" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D4800" t="n">
         <v>3</v>
@@ -86835,16 +86835,16 @@
     <row r="4801">
       <c r="A4801" t="inlineStr">
         <is>
-          <t>2027/01/02</t>
+          <t>2027/01/01</t>
         </is>
       </c>
       <c r="B4801" t="inlineStr">
         <is>
-          <t>土</t>
+          <t>金</t>
         </is>
       </c>
       <c r="C4801" t="n">
-        <v>1</v>
+        <v>19</v>
       </c>
       <c r="D4801" t="n">
         <v>3</v>
@@ -86862,7 +86862,7 @@
         </is>
       </c>
       <c r="C4802" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="D4802" t="n">
         <v>3</v>
@@ -86880,7 +86880,7 @@
         </is>
       </c>
       <c r="C4803" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="D4803" t="n">
         <v>3</v>
@@ -86898,10 +86898,10 @@
         </is>
       </c>
       <c r="C4804" t="n">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="D4804" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="4805">
@@ -86916,7 +86916,7 @@
         </is>
       </c>
       <c r="C4805" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D4805" t="n">
         <v>2</v>
@@ -86934,7 +86934,7 @@
         </is>
       </c>
       <c r="C4806" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D4806" t="n">
         <v>2</v>
@@ -86952,7 +86952,7 @@
         </is>
       </c>
       <c r="C4807" t="n">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="D4807" t="n">
         <v>2</v>
@@ -86961,16 +86961,16 @@
     <row r="4808">
       <c r="A4808" t="inlineStr">
         <is>
-          <t>2027/01/03</t>
+          <t>2027/01/02</t>
         </is>
       </c>
       <c r="B4808" t="inlineStr">
         <is>
-          <t>日</t>
+          <t>土</t>
         </is>
       </c>
       <c r="C4808" t="n">
-        <v>1</v>
+        <v>22</v>
       </c>
       <c r="D4808" t="n">
         <v>2</v>
@@ -86988,10 +86988,10 @@
         </is>
       </c>
       <c r="C4809" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D4809" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="4810">
@@ -87006,7 +87006,7 @@
         </is>
       </c>
       <c r="C4810" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="D4810" t="n">
         <v>3</v>
@@ -87024,7 +87024,7 @@
         </is>
       </c>
       <c r="C4811" t="n">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="D4811" t="n">
         <v>3</v>
@@ -87042,7 +87042,7 @@
         </is>
       </c>
       <c r="C4812" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D4812" t="n">
         <v>3</v>
@@ -87060,7 +87060,7 @@
         </is>
       </c>
       <c r="C4813" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D4813" t="n">
         <v>3</v>
@@ -87078,7 +87078,7 @@
         </is>
       </c>
       <c r="C4814" t="n">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="D4814" t="n">
         <v>3</v>
@@ -87087,16 +87087,16 @@
     <row r="4815">
       <c r="A4815" t="inlineStr">
         <is>
-          <t>2027/01/04</t>
+          <t>2027/01/03</t>
         </is>
       </c>
       <c r="B4815" t="inlineStr">
         <is>
-          <t>月</t>
+          <t>日</t>
         </is>
       </c>
       <c r="C4815" t="n">
-        <v>2</v>
+        <v>22</v>
       </c>
       <c r="D4815" t="n">
         <v>3</v>
@@ -87114,10 +87114,10 @@
         </is>
       </c>
       <c r="C4816" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D4816" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="4817">
@@ -87132,7 +87132,7 @@
         </is>
       </c>
       <c r="C4817" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="D4817" t="n">
         <v>4</v>
@@ -87150,10 +87150,10 @@
         </is>
       </c>
       <c r="C4818" t="n">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="D4818" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="4819">
@@ -87168,7 +87168,7 @@
         </is>
       </c>
       <c r="C4819" t="n">
-        <v>22</v>
+        <v>13</v>
       </c>
       <c r="D4819" t="n">
         <v>3</v>
@@ -87177,16 +87177,16 @@
     <row r="4820">
       <c r="A4820" t="inlineStr">
         <is>
-          <t>2027/01/05</t>
+          <t>2027/01/04</t>
         </is>
       </c>
       <c r="B4820" t="inlineStr">
         <is>
-          <t>火</t>
+          <t>月</t>
         </is>
       </c>
       <c r="C4820" t="n">
-        <v>1</v>
+        <v>22</v>
       </c>
       <c r="D4820" t="n">
         <v>3</v>
@@ -87204,9 +87204,27 @@
         </is>
       </c>
       <c r="C4821" t="n">
+        <v>1</v>
+      </c>
+      <c r="D4821" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="4822">
+      <c r="A4822" t="inlineStr">
+        <is>
+          <t>2027/01/05</t>
+        </is>
+      </c>
+      <c r="B4822" t="inlineStr">
+        <is>
+          <t>火</t>
+        </is>
+      </c>
+      <c r="C4822" t="n">
         <v>7</v>
       </c>
-      <c r="D4821" t="n">
+      <c r="D4822" t="n">
         <v>3</v>
       </c>
     </row>

</xml_diff>